<commit_message>
Gabarit : bibliographie BibTeX (references.bib + citeproc, nocite du top 30), citations pandoc, sans mention de la CLESSN
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01445z6xKrBFqCGGPpGngyXf
</commit_message>
<xml_diff>
--- a/Data/grille_snowballing.xlsx
+++ b/Data/grille_snowballing.xlsx
@@ -2990,7 +2990,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Research in Population Economics, 6, 183-228 (réédité 2007 dans The Economics of Language, Routledge)</t>
+          <t>Research in Population Economics, 6, 183-228</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>Recensements 1971 et 1981 : effets du statut d'immigrant, de l'ethnicité française et de la compétence linguistique sur les gains ; comparaison décennale.</t>
+          <t>Recensements 1971 et 1981 : effets du statut d'immigrant, de l'ethnicité française et de la compétence linguistique sur les gains ; comparaison décennale. Réédité en 2007 dans The Economics of Language (Routledge).</t>
         </is>
       </c>
       <c r="AM18" t="n">
@@ -17522,7 +17522,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Research in Population Economics, 6, 183-228 (réédité 2007 dans The Economics of Language, Routledge)</t>
+          <t>Research in Population Economics, 6, 183-228</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -17639,7 +17639,7 @@
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>Recensements 1971 et 1981 : effets du statut d'immigrant, de l'ethnicité française et de la compétence linguistique sur les gains ; comparaison décennale.</t>
+          <t>Recensements 1971 et 1981 : effets du statut d'immigrant, de l'ethnicité française et de la compétence linguistique sur les gains ; comparaison décennale. Réédité en 2007 dans The Economics of Language (Routledge).</t>
         </is>
       </c>
       <c r="AM16" t="n">

</xml_diff>